<commit_message>
🚀 [Auto] Sincronização de dados e código
</commit_message>
<xml_diff>
--- a/avaliacoes_garantia.xlsx
+++ b/avaliacoes_garantia.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D36"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -788,15 +788,15 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Excelente produto com pós venda atencioso e competente.</t>
+          <t>Técnico educado e cordial, realizou os reparos necessários, deixando o equipamento em pleno funcionamento.</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>45954.47363185186</v>
+        <v>46077.38118149305</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>ZDhlNGM1NDAtZWMwMy00OGRlLWE0ZDktM2JlODM0YzJhMWYwOjU3MDE2</t>
+          <t>ODIxYjc4NjQtZDdiOC00MDc2LTk3YzEtNGMwNzU1ZTdkMzkxOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -806,30 +806,34 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Excelente produto com pós venda atencioso e competente.</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>45954.47363185186</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ZDhlNGM1NDAtZWMwMy00OGRlLWE0ZDktM2JlODM0YzJhMWYwOjU3MDE2</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t xml:space="preserve">Técnico 
 Ótimo relacionamento com o cliente </t>
         </is>
       </c>
-      <c r="C24" s="2" t="n">
+      <c r="C25" s="2" t="n">
         <v>46043.57604188658</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>NjBmNTZjNjctMjFmYy00ZjU4LTg0NTItZDViMWVlZTE3NDUwOjU3MDE2</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>5</v>
-      </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" s="2" t="n">
-        <v>46006.74939984953</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>ZmYzMjBkNWUtOWQ5YS00MDFiLTk2NmItZTBlMGFlNjE3YmZiOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -839,11 +843,11 @@
       </c>
       <c r="B26" t="inlineStr"/>
       <c r="C26" s="2" t="n">
-        <v>45114.58134109954</v>
+        <v>46006.74939984953</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>MzA4YThhOWQtYjY4NS00MGZmLWE1NWItNjEwMDM4N2M1MjFiOjU3MDE2</t>
+          <t>ZmYzMjBkNWUtOWQ5YS00MDFiLTk2NmItZTBlMGFlNjE3YmZiOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -853,11 +857,11 @@
       </c>
       <c r="B27" t="inlineStr"/>
       <c r="C27" s="2" t="n">
-        <v>46006.64905208333</v>
+        <v>45114.58134109954</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>YmIzNjc4MmUtMjk5Mi00NTY3LWE5ZTEtY2VkYTU4MWM3N2NlOjU3MDE2</t>
+          <t>MzA4YThhOWQtYjY4NS00MGZmLWE1NWItNjEwMDM4N2M1MjFiOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -867,11 +871,11 @@
       </c>
       <c r="B28" t="inlineStr"/>
       <c r="C28" s="2" t="n">
-        <v>45895.62649680555</v>
+        <v>46006.64905208333</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NjMzNDFkZTQtNWEwYi00MGVhLWE0YTMtZDEzMmM1YjFjNmUyOjU3MDE2</t>
+          <t>YmIzNjc4MmUtMjk5Mi00NTY3LWE5ZTEtY2VkYTU4MWM3N2NlOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -879,17 +883,13 @@
       <c r="A29" t="n">
         <v>5</v>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>O equipamento agora está funcionando perfeitamente. Ainda não testamos para a esterilização do nosso produto. Mas acredito que vai da tudo certo.</t>
-        </is>
-      </c>
+      <c r="B29" t="inlineStr"/>
       <c r="C29" s="2" t="n">
-        <v>45954.49367453704</v>
+        <v>45895.62649680555</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>ZjIwMzgwNmItMDdmNy00OWM3LWIxMzEtYTVhZjkwNDM0OGQzOjU3MDE2</t>
+          <t>NjMzNDFkZTQtNWEwYi00MGVhLWE0YTMtZDEzMmM1YjFjNmUyOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -899,65 +899,69 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parece que vocês estão dando um rumo melhor no atendimento </t>
+          <t>O equipamento agora está funcionando perfeitamente. Ainda não testamos para a esterilização do nosso produto. Mas acredito que vai da tudo certo.</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>45919.58513085648</v>
+        <v>45954.49367453704</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NzA2MGY5NmYtZmUwZi00NTc2LTlmMDAtZjMzM2NjYzJmYWI1OjU3MDE2</t>
+          <t>ZjIwMzgwNmItMDdmNy00OWM3LWIxMzEtYTVhZjkwNDM0OGQzOjU3MDE2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pelo q.acompanhei ele fez o serviço mas uma das geladeiras continua sem baixar a temperatura ela chega no mínimo 10 graus </t>
+          <t xml:space="preserve">Parece que vocês estão dando um rumo melhor no atendimento </t>
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>45897.70520351852</v>
+        <v>45919.58513085648</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>ZjJlMGMyZjMtOWY2Yy00Yzc4LTllZmItMGM5MDE5ZjRjZmU1OjU3MDE2</t>
+          <t>NzA2MGY5NmYtZmUwZi00NTc2LTlmMDAtZjMzM2NjYzJmYWI1OjU3MDE2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>O colaborador Julio Francisco fez deu aperto em uma braçadeira que estava solta além de colocar um novo parafuso, porém não trocou a gaxeta da porta pois o arrebite é diferente</t>
+          <t xml:space="preserve">Pelo q.acompanhei ele fez o serviço mas uma das geladeiras continua sem baixar a temperatura ela chega no mínimo 10 graus </t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>45982.55515303241</v>
+        <v>45897.70520351852</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>OTc0ZmNmYTQtZTVjNi00MWQzLWI4OTQtNDI4YjYxYzcxMDRjOjU3MDE2</t>
+          <t>ZjJlMGMyZjMtOWY2Yy00Yzc4LTllZmItMGM5MDE5ZjRjZmU1OjU3MDE2</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>5</v>
-      </c>
-      <c r="B33" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>O colaborador Julio Francisco fez deu aperto em uma braçadeira que estava solta além de colocar um novo parafuso, porém não trocou a gaxeta da porta pois o arrebite é diferente</t>
+        </is>
+      </c>
       <c r="C33" s="2" t="n">
-        <v>45897.70435114583</v>
+        <v>45982.55515303241</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ZGZmYTBjMjEtN2ZiOC00NTUzLTg2NDEtODg4ZWJlNTI2ZWRjOjU3MDE2</t>
+          <t>OTc0ZmNmYTQtZTVjNi00MWQzLWI4OTQtNDI4YjYxYzcxMDRjOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -967,11 +971,11 @@
       </c>
       <c r="B34" t="inlineStr"/>
       <c r="C34" s="2" t="n">
-        <v>45940.6359195949</v>
+        <v>45897.70435114583</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ZDljNWUxNGUtNDI1OS00ZTZhLWEzZmMtODlmMmZkMzNlMzBjOjU3MDE2</t>
+          <t>ZGZmYTBjMjEtN2ZiOC00NTUzLTg2NDEtODg4ZWJlNTI2ZWRjOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -979,17 +983,13 @@
       <c r="A35" t="n">
         <v>5</v>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Colaborador muito atencioso. </t>
-        </is>
-      </c>
+      <c r="B35" t="inlineStr"/>
       <c r="C35" s="2" t="n">
-        <v>45918.57075675926</v>
+        <v>45940.6359195949</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Yzg4MTJkNjgtYzBhOS00ODY0LWE3NmItMjMzN2ZkMWUwODA2OjU3MDE2</t>
+          <t>ZDljNWUxNGUtNDI1OS00ZTZhLWEzZmMtODlmMmZkMzNlMzBjOjU3MDE2</t>
         </is>
       </c>
     </row>
@@ -997,11 +997,29 @@
       <c r="A36" t="n">
         <v>5</v>
       </c>
-      <c r="B36" t="inlineStr"/>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Colaborador muito atencioso. </t>
+        </is>
+      </c>
       <c r="C36" s="2" t="n">
+        <v>45918.57075675926</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Yzg4MTJkNjgtYzBhOS00ODY0LWE3NmItMjMzN2ZkMWUwODA2OjU3MDE2</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" s="2" t="n">
         <v>45940.63159275463</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>NzYxOTRkMzgtZDQwNy00ODM5LWI5NDctYzJkMTczZDkzZGQzOjU3MDE2</t>
         </is>

</xml_diff>